<commit_message>
Fix old site names and rebuild all workbooks
</commit_message>
<xml_diff>
--- a/data/competitions/93/workbook.xlsx
+++ b/data/competitions/93/workbook.xlsx
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C13" t="n">
         <v>51</v>
@@ -615,13 +615,13 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>-23.21428571</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -653,7 +653,7 @@
         <v>52</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>35.71428571</v>
+        <v>33.05785124</v>
       </c>
     </row>
     <row r="17">
@@ -669,7 +669,7 @@
         <v>45</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-58.92857143</v>
+        <v>-54.54545455</v>
       </c>
     </row>
     <row r="19">
@@ -726,10 +726,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C25" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26">
@@ -739,13 +739,13 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>360.6557377</v>
+        <v>442.85714286</v>
       </c>
     </row>
     <row r="27">
@@ -771,7 +771,7 @@
         <v>53</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>111.47540984</v>
+        <v>48.57142857</v>
       </c>
     </row>
     <row r="29">
@@ -787,7 +787,7 @@
         <v>36</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>-468.85245902</v>
+        <v>-471.42857143</v>
       </c>
     </row>
     <row r="31">
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C43" t="n">
         <v>59</v>
@@ -934,7 +934,7 @@
         <v>58</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>-45.87155963</v>
+        <v>-45.04504505</v>
       </c>
     </row>
     <row r="45">
@@ -950,7 +950,7 @@
         <v>63</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>128.44036697</v>
+        <v>126.12612613</v>
       </c>
     </row>
     <row r="46">
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>-42.20183486</v>
+        <v>-67.56756756999999</v>
       </c>
     </row>
     <row r="47">
@@ -982,7 +982,7 @@
         <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>-54.12844037</v>
+        <v>-53.15315315</v>
       </c>
     </row>
     <row r="49">
@@ -4106,7 +4106,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -4182,7 +4182,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -5284,7 +5284,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Lobby/Piano</t>
+          <t>Exposition/Piano</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Lobby/Piano</t>
+          <t>Exposition/Piano</t>
         </is>
       </c>
       <c r="H37" t="n">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H60" t="n">
@@ -6348,7 +6348,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H115" t="n">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H116" t="n">
@@ -8666,7 +8666,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H122" t="n">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H123" t="n">
@@ -8818,7 +8818,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H126" t="n">
@@ -9046,7 +9046,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H132" t="n">
@@ -9084,7 +9084,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Kitchen/Trophy</t>
+          <t>Kitchen/Dining</t>
         </is>
       </c>
       <c r="H133" t="n">
@@ -12010,7 +12010,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H210" t="n">
@@ -12086,7 +12086,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H212" t="n">
@@ -12314,7 +12314,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H218" t="n">
@@ -12352,7 +12352,7 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H219" t="n">
@@ -12656,7 +12656,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H227" t="n">
@@ -12694,7 +12694,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H228" t="n">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Armory/Archives</t>
+          <t>Archives/Armory</t>
         </is>
       </c>
       <c r="H229" t="n">
@@ -78988,7 +78988,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Chalet | Europe MENA League 2026 Challenger Series | 12 games | 112 rounds</t>
+          <t>Chalet | Europe MENA League 2026 Challenger Series | 12 games | 121 rounds</t>
         </is>
       </c>
     </row>
@@ -79056,16 +79056,16 @@
         </is>
       </c>
       <c r="H4" s="1" t="n">
-        <v>35.71428571</v>
+        <v>33.05785124</v>
       </c>
       <c r="I4" s="1" t="n">
-        <v>-23.21428571</v>
+        <v>0</v>
       </c>
       <c r="J4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K4" s="1" t="n">
-        <v>-58.92857143</v>
+        <v>-54.54545455</v>
       </c>
     </row>
     <row r="5">
@@ -79121,7 +79121,7 @@
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>2</v>
@@ -79133,7 +79133,7 @@
         <v>13</v>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J6" t="n">
         <v>12</v>
@@ -79158,7 +79158,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -79170,7 +79170,7 @@
         <v>4</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J7" t="n">
         <v>2</v>
@@ -79232,7 +79232,7 @@
         <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -79244,7 +79244,7 @@
         <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -79269,7 +79269,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>3</v>
@@ -79281,7 +79281,7 @@
         <v>12</v>
       </c>
       <c r="I10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J10" t="n">
         <v>13</v>
@@ -79380,7 +79380,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -79392,7 +79392,7 @@
         <v>42</v>
       </c>
       <c r="I13" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J13" t="n">
         <v>42</v>
@@ -79639,7 +79639,7 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -79651,7 +79651,7 @@
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -79898,7 +79898,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -79910,7 +79910,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -80094,16 +80094,16 @@
         </is>
       </c>
       <c r="H33" s="1" t="n">
-        <v>35.71428571</v>
+        <v>33.05785124</v>
       </c>
       <c r="I33" s="1" t="n">
-        <v>-23.21428571</v>
+        <v>0</v>
       </c>
       <c r="J33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K33" s="1" t="n">
-        <v>-58.92857143</v>
+        <v>-54.54545455</v>
       </c>
     </row>
     <row r="34">
@@ -80122,7 +80122,7 @@
         <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
         <v>2</v>
@@ -80134,7 +80134,7 @@
         <v>3</v>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J34" t="n">
         <v>2</v>
@@ -80233,7 +80233,7 @@
         <v>2</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>2</v>
@@ -80245,7 +80245,7 @@
         <v>21</v>
       </c>
       <c r="I37" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J37" t="n">
         <v>21</v>
@@ -80307,7 +80307,7 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
         <v>2</v>
@@ -80319,7 +80319,7 @@
         <v>42</v>
       </c>
       <c r="I39" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J39" t="n">
         <v>43</v>
@@ -80418,7 +80418,7 @@
         <v>3</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -80430,7 +80430,7 @@
         <v>3</v>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -80936,7 +80936,7 @@
         <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -80948,7 +80948,7 @@
         <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -81209,7 +81209,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Border | Europe MENA League 2026 Challenger Series | 6 games | 61 rounds</t>
+          <t>Border | Europe MENA League 2026 Challenger Series | 6 games | 70 rounds</t>
         </is>
       </c>
     </row>
@@ -81277,14 +81277,14 @@
         </is>
       </c>
       <c r="H4" s="1" t="n">
-        <v>360.6557377</v>
+        <v>442.85714286</v>
       </c>
       <c r="I4" s="1" t="n"/>
       <c r="J4" s="1" t="n">
-        <v>-468.85245902</v>
+        <v>-471.42857143</v>
       </c>
       <c r="K4" s="1" t="n">
-        <v>111.47540984</v>
+        <v>48.57142857</v>
       </c>
     </row>
     <row r="5">
@@ -81300,7 +81300,7 @@
         <v>22</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -81312,7 +81312,7 @@
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I5" t="n">
         <v>22</v>
@@ -81337,7 +81337,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -81349,7 +81349,7 @@
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -81411,7 +81411,7 @@
         <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -81423,7 +81423,7 @@
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I8" t="n">
         <v>15</v>
@@ -81744,7 +81744,7 @@
         <v>74</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -81756,7 +81756,7 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I17" t="n">
         <v>74</v>
@@ -82128,14 +82128,14 @@
         </is>
       </c>
       <c r="H28" s="1" t="n">
-        <v>360.6557377</v>
+        <v>442.85714286</v>
       </c>
       <c r="I28" s="1" t="n"/>
       <c r="J28" s="1" t="n">
-        <v>-468.85245902</v>
+        <v>-471.42857143</v>
       </c>
       <c r="K28" s="1" t="n">
-        <v>111.47540984</v>
+        <v>48.57142857</v>
       </c>
     </row>
     <row r="29">
@@ -82188,7 +82188,7 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
@@ -82200,7 +82200,7 @@
         <v>3</v>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -82225,7 +82225,7 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
@@ -82237,7 +82237,7 @@
         <v>2</v>
       </c>
       <c r="H31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -82262,7 +82262,7 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
@@ -82274,7 +82274,7 @@
         <v>1</v>
       </c>
       <c r="H32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
@@ -82336,7 +82336,7 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -82348,7 +82348,7 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -82521,7 +82521,7 @@
         <v>11</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
@@ -82533,7 +82533,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I39" t="n">
         <v>11</v>
@@ -85421,7 +85421,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Consulate | Europe MENA League 2026 Challenger Series | 10 games | 109 rounds</t>
+          <t>Consulate | Europe MENA League 2026 Challenger Series | 10 games | 111 rounds</t>
         </is>
       </c>
     </row>
@@ -85489,16 +85489,16 @@
         </is>
       </c>
       <c r="H4" s="1" t="n">
-        <v>128.44036697</v>
+        <v>126.12612613</v>
       </c>
       <c r="I4" s="1" t="n">
-        <v>-45.87155963</v>
+        <v>-45.04504505</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>-42.20183486</v>
+        <v>-67.56756756999999</v>
       </c>
       <c r="K4" s="1" t="n">
-        <v>-54.12844037</v>
+        <v>-53.15315315</v>
       </c>
     </row>
     <row r="5">
@@ -85890,7 +85890,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -85902,7 +85902,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -86601,16 +86601,16 @@
         </is>
       </c>
       <c r="H35" s="1" t="n">
-        <v>128.44036697</v>
+        <v>126.12612613</v>
       </c>
       <c r="I35" s="1" t="n">
-        <v>-45.87155963</v>
+        <v>-45.04504505</v>
       </c>
       <c r="J35" s="1" t="n">
-        <v>-42.20183486</v>
+        <v>-67.56756756999999</v>
       </c>
       <c r="K35" s="1" t="n">
-        <v>-54.12844037</v>
+        <v>-53.15315315</v>
       </c>
     </row>
     <row r="36">
@@ -87298,7 +87298,7 @@
         <v>2</v>
       </c>
       <c r="F54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G54" t="n">
         <v>0</v>
@@ -87310,7 +87310,7 @@
         <v>2</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>

</xml_diff>